<commit_message>
TAREFA MENU PRINCIPAL CONCLUÍDA
</commit_message>
<xml_diff>
--- a/Basico/32 - Procv Aproximado 1.xlsx
+++ b/Basico/32 - Procv Aproximado 1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\Luiz Henrique Vidal Araujo - Excel completo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Basico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD5B61C-6374-473A-8C2F-411AAF9C4A6C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBB6E84A-66D0-4C9C-9CA3-125CAE6CCD58}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="15360" windowHeight="7425" firstSheet="24" activeTab="30" xr2:uid="{A5E3398E-808E-49BA-92C6-AB43937C9D3D}"/>
   </bookViews>
@@ -1783,6 +1783,15 @@
     <xf numFmtId="14" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="169" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1888,26 +1897,17 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2301,18 +2301,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="90" t="s">
+      <c r="A1" s="93" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
+      <c r="B1" s="93"/>
+      <c r="C1" s="93"/>
+      <c r="D1" s="93"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="91" t="s">
+      <c r="A2" s="94" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="92" t="s">
+      <c r="B2" s="95" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="2">
@@ -2324,8 +2324,8 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="91"/>
-      <c r="B3" s="92"/>
+      <c r="A3" s="94"/>
+      <c r="B3" s="95"/>
       <c r="C3" s="3">
         <v>0.1</v>
       </c>
@@ -2335,8 +2335,8 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="91"/>
-      <c r="B4" s="92"/>
+      <c r="A4" s="94"/>
+      <c r="B4" s="95"/>
       <c r="C4">
         <v>2.58</v>
       </c>
@@ -2346,8 +2346,8 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="91"/>
-      <c r="B5" s="92"/>
+      <c r="A5" s="94"/>
+      <c r="B5" s="95"/>
       <c r="C5" s="4">
         <v>1000</v>
       </c>
@@ -2357,8 +2357,8 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="91"/>
-      <c r="B6" s="92"/>
+      <c r="A6" s="94"/>
+      <c r="B6" s="95"/>
       <c r="C6" s="5">
         <v>42567</v>
       </c>
@@ -2368,8 +2368,8 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="91"/>
-      <c r="B7" s="92"/>
+      <c r="A7" s="94"/>
+      <c r="B7" s="95"/>
       <c r="C7" s="6" t="s">
         <v>0</v>
       </c>
@@ -2394,11 +2394,11 @@
   <sheetFormatPr defaultColWidth="18.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="100" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="98"/>
-      <c r="C1" s="99"/>
+      <c r="B1" s="101"/>
+      <c r="C1" s="102"/>
     </row>
     <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
@@ -2521,11 +2521,11 @@
   <sheetFormatPr defaultColWidth="18.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="99" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
     </row>
     <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
@@ -2685,11 +2685,11 @@
   <sheetFormatPr defaultColWidth="18.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="99" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
     </row>
     <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
@@ -2832,15 +2832,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="103" t="s">
         <v>113</v>
       </c>
-      <c r="B1" s="100"/>
-      <c r="C1" s="100"/>
-      <c r="D1" s="100"/>
-      <c r="E1" s="100"/>
-      <c r="F1" s="100"/>
-      <c r="G1" s="100"/>
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
+      <c r="D1" s="103"/>
+      <c r="E1" s="103"/>
+      <c r="F1" s="103"/>
+      <c r="G1" s="103"/>
     </row>
     <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
@@ -3148,13 +3148,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="103" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
+      <c r="B1" s="104"/>
+      <c r="C1" s="104"/>
+      <c r="D1" s="104"/>
+      <c r="E1" s="104"/>
     </row>
     <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
@@ -3356,10 +3356,10 @@
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
-      <c r="C13" s="102" t="s">
+      <c r="C13" s="105" t="s">
         <v>146</v>
       </c>
-      <c r="D13" s="103"/>
+      <c r="D13" s="106"/>
       <c r="E13" s="43">
         <f>SUM(E3:E12)</f>
         <v>12606</v>
@@ -3384,11 +3384,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="105" t="s">
         <v>148</v>
       </c>
-      <c r="B1" s="104"/>
-      <c r="C1" s="103"/>
+      <c r="B1" s="107"/>
+      <c r="C1" s="106"/>
     </row>
     <row r="2" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="39" t="s">
@@ -3511,12 +3511,12 @@
   <sheetFormatPr defaultColWidth="18.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="105" t="s">
+      <c r="A1" s="108" t="s">
         <v>159</v>
       </c>
-      <c r="B1" s="106"/>
-      <c r="C1" s="106"/>
-      <c r="D1" s="107"/>
+      <c r="B1" s="109"/>
+      <c r="C1" s="109"/>
+      <c r="D1" s="110"/>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
@@ -3635,14 +3635,14 @@
   <sheetFormatPr defaultColWidth="18.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="105" t="s">
+      <c r="A1" s="108" t="s">
         <v>171</v>
       </c>
-      <c r="B1" s="106"/>
-      <c r="C1" s="106"/>
-      <c r="D1" s="106"/>
-      <c r="E1" s="106"/>
-      <c r="F1" s="107"/>
+      <c r="B1" s="109"/>
+      <c r="C1" s="109"/>
+      <c r="D1" s="109"/>
+      <c r="E1" s="109"/>
+      <c r="F1" s="110"/>
     </row>
     <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
@@ -3929,40 +3929,40 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D15" s="101" t="s">
+      <c r="D15" s="104" t="s">
         <v>177</v>
       </c>
-      <c r="E15" s="101"/>
+      <c r="E15" s="104"/>
       <c r="F15" s="26">
         <f>SUM(F3:F14)</f>
         <v>8669.24</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D16" s="101" t="s">
+      <c r="D16" s="104" t="s">
         <v>178</v>
       </c>
-      <c r="E16" s="101"/>
+      <c r="E16" s="104"/>
       <c r="F16" s="26">
         <f>AVERAGE(F3:F14)</f>
         <v>722.43666666666661</v>
       </c>
     </row>
     <row r="17" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D17" s="101" t="s">
+      <c r="D17" s="104" t="s">
         <v>179</v>
       </c>
-      <c r="E17" s="101"/>
+      <c r="E17" s="104"/>
       <c r="F17" s="26">
         <f>MAX(F3:F14)</f>
         <v>1670.3999999999999</v>
       </c>
     </row>
     <row r="18" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D18" s="101" t="s">
+      <c r="D18" s="104" t="s">
         <v>180</v>
       </c>
-      <c r="E18" s="101"/>
+      <c r="E18" s="104"/>
       <c r="F18" s="26">
         <f>MIN(F3:F14)</f>
         <v>160.5</v>
@@ -3990,14 +3990,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="111" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
+      <c r="B1" s="111"/>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="111"/>
+      <c r="F1" s="111"/>
     </row>
     <row r="2" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
@@ -4145,60 +4145,60 @@
   <sheetFormatPr defaultColWidth="18.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="111" t="s">
         <v>206</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
+      <c r="B1" s="111"/>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="51" t="s">
         <v>208</v>
       </c>
-      <c r="B2" s="109" t="s">
+      <c r="B2" s="112" t="s">
         <v>210</v>
       </c>
-      <c r="C2" s="110"/>
-      <c r="D2" s="111"/>
+      <c r="C2" s="113"/>
+      <c r="D2" s="114"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="51" t="s">
         <v>43</v>
       </c>
-      <c r="B3" s="112">
+      <c r="B3" s="115">
         <v>5144230</v>
       </c>
-      <c r="C3" s="113"/>
-      <c r="D3" s="114"/>
+      <c r="C3" s="116"/>
+      <c r="D3" s="117"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="51" t="s">
         <v>207</v>
       </c>
-      <c r="B4" s="109" t="s">
+      <c r="B4" s="112" t="s">
         <v>211</v>
       </c>
-      <c r="C4" s="110"/>
-      <c r="D4" s="111"/>
+      <c r="C4" s="113"/>
+      <c r="D4" s="114"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="51" t="s">
         <v>154</v>
       </c>
-      <c r="B5" s="115">
+      <c r="B5" s="118">
         <v>33337878</v>
       </c>
-      <c r="C5" s="116"/>
-      <c r="D5" s="117"/>
+      <c r="C5" s="119"/>
+      <c r="D5" s="120"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="108" t="s">
+      <c r="A7" s="111" t="s">
         <v>205</v>
       </c>
-      <c r="B7" s="108"/>
-      <c r="C7" s="108"/>
-      <c r="D7" s="108"/>
+      <c r="B7" s="111"/>
+      <c r="C7" s="111"/>
+      <c r="D7" s="111"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="38" t="s">
@@ -4290,10 +4290,10 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B15" s="102" t="s">
+      <c r="B15" s="105" t="s">
         <v>209</v>
       </c>
-      <c r="C15" s="103"/>
+      <c r="C15" s="106"/>
       <c r="D15" s="26">
         <f>SUM(D9:D13)</f>
         <v>42790</v>
@@ -4324,10 +4324,10 @@
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B18" s="102" t="s">
+      <c r="B18" s="105" t="s">
         <v>200</v>
       </c>
-      <c r="C18" s="103"/>
+      <c r="C18" s="106"/>
       <c r="D18" s="26">
         <f>SUM(D15:D17)</f>
         <v>52631.7</v>
@@ -4555,15 +4555,15 @@
   <sheetFormatPr defaultColWidth="18.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="118" t="s">
+      <c r="A1" s="121" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
+      <c r="B1" s="122"/>
+      <c r="C1" s="122"/>
+      <c r="D1" s="122"/>
+      <c r="E1" s="122"/>
+      <c r="F1" s="122"/>
+      <c r="G1" s="122"/>
     </row>
     <row r="2" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A2" s="55" t="s">
@@ -4826,14 +4826,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="103" t="s">
         <v>234</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="D1" s="105" t="s">
+      <c r="B1" s="104"/>
+      <c r="D1" s="108" t="s">
         <v>237</v>
       </c>
-      <c r="E1" s="107"/>
+      <c r="E1" s="110"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="40"/>
@@ -4957,23 +4957,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="103" t="s">
         <v>242</v>
       </c>
-      <c r="B1" s="100"/>
-      <c r="C1" s="100"/>
-      <c r="D1" s="100"/>
-      <c r="E1" s="100"/>
-      <c r="G1" s="100" t="s">
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
+      <c r="D1" s="103"/>
+      <c r="E1" s="103"/>
+      <c r="G1" s="103" t="s">
         <v>237</v>
       </c>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
+      <c r="H1" s="104"/>
+      <c r="I1" s="104"/>
+      <c r="J1" s="104"/>
+      <c r="K1" s="104"/>
+      <c r="L1" s="104"/>
+      <c r="M1" s="104"/>
+      <c r="N1" s="104"/>
     </row>
     <row r="2" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="48" t="s">
@@ -4987,20 +4987,20 @@
       <c r="E2" s="48" t="s">
         <v>245</v>
       </c>
-      <c r="G2" s="120" t="s">
+      <c r="G2" s="123" t="s">
         <v>246</v>
       </c>
-      <c r="H2" s="120"/>
+      <c r="H2" s="123"/>
       <c r="I2" s="7"/>
-      <c r="J2" s="101" t="s">
+      <c r="J2" s="104" t="s">
         <v>247</v>
       </c>
-      <c r="K2" s="101"/>
+      <c r="K2" s="104"/>
       <c r="L2" s="7"/>
-      <c r="M2" s="101" t="s">
+      <c r="M2" s="104" t="s">
         <v>248</v>
       </c>
-      <c r="N2" s="101"/>
+      <c r="N2" s="104"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
@@ -5237,18 +5237,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="121" t="s">
+      <c r="A1" s="124" t="s">
         <v>257</v>
       </c>
-      <c r="B1" s="122"/>
-      <c r="C1" s="122"/>
-      <c r="D1" s="122"/>
-      <c r="E1" s="123"/>
-      <c r="G1" s="108" t="s">
+      <c r="B1" s="125"/>
+      <c r="C1" s="125"/>
+      <c r="D1" s="125"/>
+      <c r="E1" s="126"/>
+      <c r="G1" s="111" t="s">
         <v>263</v>
       </c>
-      <c r="H1" s="108"/>
-      <c r="I1" s="108"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
     </row>
     <row r="2" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
@@ -5735,18 +5735,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="103" t="s">
         <v>273</v>
       </c>
-      <c r="B1" s="100"/>
-      <c r="C1" s="100"/>
-      <c r="D1" s="100"/>
-      <c r="F1" s="100" t="s">
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
+      <c r="D1" s="103"/>
+      <c r="F1" s="103" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="100"/>
-      <c r="H1" s="100"/>
-      <c r="I1" s="100"/>
+      <c r="G1" s="103"/>
+      <c r="H1" s="103"/>
+      <c r="I1" s="103"/>
     </row>
     <row r="2" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
@@ -5946,11 +5946,11 @@
       <c r="D9" s="41">
         <v>444.69</v>
       </c>
-      <c r="F9" s="101" t="s">
+      <c r="F9" s="104" t="s">
         <v>293</v>
       </c>
-      <c r="G9" s="101"/>
-      <c r="H9" s="101"/>
+      <c r="G9" s="104"/>
+      <c r="H9" s="104"/>
       <c r="I9" s="53">
         <v>0.1</v>
       </c>
@@ -5968,11 +5968,11 @@
       <c r="D10" s="41">
         <v>245.9</v>
       </c>
-      <c r="F10" s="101" t="s">
+      <c r="F10" s="104" t="s">
         <v>294</v>
       </c>
-      <c r="G10" s="101"/>
-      <c r="H10" s="101"/>
+      <c r="G10" s="104"/>
+      <c r="H10" s="104"/>
       <c r="I10" s="43">
         <f>SUM(I3:I7)</f>
         <v>854.57200000000012</v>
@@ -6097,13 +6097,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="103" t="s">
         <v>303</v>
       </c>
-      <c r="B1" s="100"/>
-      <c r="C1" s="100"/>
-      <c r="D1" s="100"/>
-      <c r="E1" s="100"/>
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
+      <c r="D1" s="103"/>
+      <c r="E1" s="103"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="60" t="s">
@@ -6113,10 +6113,10 @@
         <v>100</v>
       </c>
       <c r="C2" s="7"/>
-      <c r="D2" s="102" t="s">
+      <c r="D2" s="105" t="s">
         <v>296</v>
       </c>
-      <c r="E2" s="103"/>
+      <c r="E2" s="106"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="45" t="s">
@@ -6233,10 +6233,10 @@
         <v>20184</v>
       </c>
       <c r="C10" s="7"/>
-      <c r="D10" s="102" t="s">
+      <c r="D10" s="105" t="s">
         <v>302</v>
       </c>
-      <c r="E10" s="103"/>
+      <c r="E10" s="106"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="45" t="s">
@@ -6439,12 +6439,12 @@
   <sheetFormatPr defaultColWidth="18.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="111" t="s">
         <v>305</v>
       </c>
-      <c r="B1" s="124"/>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
+      <c r="B1" s="127"/>
+      <c r="C1" s="127"/>
+      <c r="D1" s="127"/>
     </row>
     <row r="2" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
@@ -6610,11 +6610,11 @@
   <sheetFormatPr defaultColWidth="18.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="103" t="s">
         <v>316</v>
       </c>
-      <c r="B1" s="100"/>
-      <c r="C1" s="100"/>
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="61" t="s">
@@ -6741,11 +6741,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="105" t="s">
+      <c r="A1" s="108" t="s">
         <v>325</v>
       </c>
-      <c r="B1" s="106"/>
-      <c r="C1" s="107"/>
+      <c r="B1" s="109"/>
+      <c r="C1" s="110"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="61" t="s">
@@ -6885,17 +6885,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="111" t="s">
         <v>342</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="F1" s="100" t="s">
+      <c r="B1" s="111"/>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
+      <c r="F1" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="G1" s="100"/>
-      <c r="H1" s="100"/>
+      <c r="G1" s="103"/>
+      <c r="H1" s="103"/>
     </row>
     <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="67" t="s">
@@ -7144,12 +7144,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="96" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="93"/>
-      <c r="C1" s="93"/>
-      <c r="D1" s="93"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
@@ -7256,16 +7256,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="111" t="s">
         <v>414</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="108"/>
+      <c r="B1" s="111"/>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="111"/>
+      <c r="F1" s="111"/>
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
       <c r="J1" s="77"/>
       <c r="K1" s="77"/>
       <c r="L1" s="77"/>
@@ -7694,11 +7694,11 @@
       <c r="Q14" s="83"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A15" s="125" t="s">
+      <c r="A15" s="130" t="s">
         <v>408</v>
       </c>
-      <c r="B15" s="125"/>
-      <c r="C15" s="125"/>
+      <c r="B15" s="130"/>
+      <c r="C15" s="130"/>
       <c r="J15" s="84"/>
       <c r="K15" s="84"/>
       <c r="L15" s="84"/>
@@ -7712,10 +7712,10 @@
       <c r="A16" s="76" t="s">
         <v>409</v>
       </c>
-      <c r="B16" s="126" t="s">
+      <c r="B16" s="131" t="s">
         <v>400</v>
       </c>
-      <c r="C16" s="126"/>
+      <c r="C16" s="131"/>
       <c r="J16" s="85"/>
       <c r="K16" s="89"/>
       <c r="L16" s="89"/>
@@ -7729,11 +7729,11 @@
       <c r="A17" s="76" t="s">
         <v>410</v>
       </c>
-      <c r="B17" s="127">
+      <c r="B17" s="128">
         <f>VLOOKUP($B$16,$A$3:$H$13,2,FALSE)</f>
         <v>32240</v>
       </c>
-      <c r="C17" s="127"/>
+      <c r="C17" s="128"/>
       <c r="J17" s="85"/>
       <c r="K17" s="87"/>
       <c r="L17" s="87"/>
@@ -7747,11 +7747,11 @@
       <c r="A18" s="76" t="s">
         <v>411</v>
       </c>
-      <c r="B18" s="127" t="str">
+      <c r="B18" s="128" t="str">
         <f>VLOOKUP($B$16,$A$3:$H$13,3,FALSE)</f>
         <v>M</v>
       </c>
-      <c r="C18" s="127"/>
+      <c r="C18" s="128"/>
       <c r="J18" s="85"/>
       <c r="K18" s="87"/>
       <c r="L18" s="87"/>
@@ -7765,11 +7765,11 @@
       <c r="A19" s="76" t="s">
         <v>208</v>
       </c>
-      <c r="B19" s="127" t="str">
+      <c r="B19" s="128" t="str">
         <f>VLOOKUP($B$16,$A$3:$H$13,4,FALSE)</f>
         <v>Av. João Bosco, 415</v>
       </c>
-      <c r="C19" s="127"/>
+      <c r="C19" s="128"/>
       <c r="J19" s="85"/>
       <c r="K19" s="87"/>
       <c r="L19" s="87"/>
@@ -7783,11 +7783,11 @@
       <c r="A20" s="76" t="s">
         <v>412</v>
       </c>
-      <c r="B20" s="127" t="str">
+      <c r="B20" s="128" t="str">
         <f>VLOOKUP($B$16,$A$3:$H$13,5,FALSE)</f>
         <v>Leme</v>
       </c>
-      <c r="C20" s="127"/>
+      <c r="C20" s="128"/>
       <c r="J20" s="85"/>
       <c r="K20" s="87"/>
       <c r="L20" s="87"/>
@@ -7801,11 +7801,11 @@
       <c r="A21" s="76" t="s">
         <v>207</v>
       </c>
-      <c r="B21" s="127" t="str">
+      <c r="B21" s="128" t="str">
         <f>VLOOKUP($B$16,$A$3:$H$13,6,FALSE)</f>
         <v>Carapícuiba</v>
       </c>
-      <c r="C21" s="127"/>
+      <c r="C21" s="128"/>
       <c r="J21" s="85"/>
       <c r="K21" s="87"/>
       <c r="L21" s="87"/>
@@ -7819,11 +7819,11 @@
       <c r="A22" s="76" t="s">
         <v>413</v>
       </c>
-      <c r="B22" s="127" t="str">
+      <c r="B22" s="128" t="str">
         <f>VLOOKUP($B$16,$A$3:$H$13,7,FALSE)</f>
         <v>SP</v>
       </c>
-      <c r="C22" s="127"/>
+      <c r="C22" s="128"/>
       <c r="J22" s="85"/>
       <c r="K22" s="87"/>
       <c r="L22" s="87"/>
@@ -7837,11 +7837,11 @@
       <c r="A23" s="76" t="s">
         <v>43</v>
       </c>
-      <c r="B23" s="128">
+      <c r="B23" s="129">
         <f>VLOOKUP($B$16,$A$3:$H$13,8,FALSE)</f>
         <v>8484012</v>
       </c>
-      <c r="C23" s="128"/>
+      <c r="C23" s="129"/>
       <c r="J23" s="85"/>
       <c r="K23" s="88"/>
       <c r="L23" s="88"/>
@@ -7873,16 +7873,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="B23:C23"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K16:L16" xr:uid="{D24E4997-11E7-43F4-98AD-8963A5EEE39C}">
@@ -7903,41 +7903,41 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="3.42578125" customWidth="1"/>
     <col min="10" max="10" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="103" t="s">
         <v>418</v>
       </c>
-      <c r="B1" s="100"/>
-      <c r="C1" s="100"/>
-      <c r="D1" s="100"/>
-      <c r="E1" s="100"/>
-      <c r="F1" s="100"/>
-      <c r="H1" s="125" t="s">
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
+      <c r="D1" s="103"/>
+      <c r="E1" s="103"/>
+      <c r="F1" s="103"/>
+      <c r="H1" s="130" t="s">
         <v>415</v>
       </c>
-      <c r="I1" s="125"/>
-      <c r="J1" s="125"/>
+      <c r="I1" s="130"/>
+      <c r="J1" s="130"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="129" t="s">
+      <c r="A2" s="90" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="129" t="s">
+      <c r="B2" s="90" t="s">
         <v>419</v>
       </c>
-      <c r="C2" s="129" t="s">
+      <c r="C2" s="90" t="s">
         <v>420</v>
       </c>
-      <c r="D2" s="129" t="s">
+      <c r="D2" s="90" t="s">
         <v>421</v>
       </c>
-      <c r="E2" s="129" t="s">
+      <c r="E2" s="90" t="s">
         <v>422</v>
       </c>
       <c r="F2" s="72" t="s">
@@ -7963,12 +7963,12 @@
       <c r="C3" s="42">
         <v>54</v>
       </c>
-      <c r="D3" s="130">
+      <c r="D3" s="91">
         <v>1.6</v>
       </c>
-      <c r="E3" s="130">
-        <f>C3/(D3*D3)</f>
-        <v>21.093749999999996</v>
+      <c r="E3" s="91">
+        <f>TRUNC(C3/(D3*D3),2)</f>
+        <v>21.09</v>
       </c>
       <c r="F3" s="45" t="str">
         <f>VLOOKUP(E3,$H$3:$J$7,3,TRUE)</f>
@@ -7988,16 +7988,16 @@
       <c r="A4" s="45" t="s">
         <v>424</v>
       </c>
-      <c r="B4" s="131">
+      <c r="B4" s="92">
         <v>28</v>
       </c>
       <c r="C4" s="42">
         <v>58</v>
       </c>
-      <c r="D4" s="130">
+      <c r="D4" s="91">
         <v>1.75</v>
       </c>
-      <c r="E4" s="130">
+      <c r="E4" s="91">
         <f t="shared" ref="E4:E13" si="0">C4/(D4*D4)</f>
         <v>18.938775510204081</v>
       </c>
@@ -8025,10 +8025,10 @@
       <c r="C5" s="42">
         <v>70</v>
       </c>
-      <c r="D5" s="130">
+      <c r="D5" s="91">
         <v>1.68</v>
       </c>
-      <c r="E5" s="130">
+      <c r="E5" s="91">
         <f t="shared" si="0"/>
         <v>24.801587301587304</v>
       </c>
@@ -8056,10 +8056,10 @@
       <c r="C6" s="42">
         <v>115</v>
       </c>
-      <c r="D6" s="130">
+      <c r="D6" s="91">
         <v>1.9</v>
       </c>
-      <c r="E6" s="130">
+      <c r="E6" s="91">
         <f t="shared" si="0"/>
         <v>31.855955678670362</v>
       </c>
@@ -8087,10 +8087,10 @@
       <c r="C7" s="42">
         <v>62</v>
       </c>
-      <c r="D7" s="130">
+      <c r="D7" s="91">
         <v>1.54</v>
       </c>
-      <c r="E7" s="130">
+      <c r="E7" s="91">
         <f t="shared" si="0"/>
         <v>26.14268848035082</v>
       </c>
@@ -8118,10 +8118,10 @@
       <c r="C8" s="42">
         <v>59</v>
       </c>
-      <c r="D8" s="130">
+      <c r="D8" s="91">
         <v>1.61</v>
       </c>
-      <c r="E8" s="130">
+      <c r="E8" s="91">
         <f t="shared" si="0"/>
         <v>22.761467535974688</v>
       </c>
@@ -8140,10 +8140,10 @@
       <c r="C9" s="42">
         <v>74</v>
       </c>
-      <c r="D9" s="130">
+      <c r="D9" s="91">
         <v>1.63</v>
       </c>
-      <c r="E9" s="130">
+      <c r="E9" s="91">
         <f t="shared" si="0"/>
         <v>27.852007979223909</v>
       </c>
@@ -8162,10 +8162,10 @@
       <c r="C10" s="42">
         <v>68</v>
       </c>
-      <c r="D10" s="130">
+      <c r="D10" s="91">
         <v>1.75</v>
       </c>
-      <c r="E10" s="130">
+      <c r="E10" s="91">
         <f t="shared" si="0"/>
         <v>22.204081632653061</v>
       </c>
@@ -8184,10 +8184,10 @@
       <c r="C11" s="42">
         <v>94</v>
       </c>
-      <c r="D11" s="130">
+      <c r="D11" s="91">
         <v>1.82</v>
       </c>
-      <c r="E11" s="130">
+      <c r="E11" s="91">
         <f t="shared" si="0"/>
         <v>28.378215191402003</v>
       </c>
@@ -8206,10 +8206,10 @@
       <c r="C12" s="42">
         <v>60</v>
       </c>
-      <c r="D12" s="130">
+      <c r="D12" s="91">
         <v>1.59</v>
       </c>
-      <c r="E12" s="130">
+      <c r="E12" s="91">
         <f t="shared" si="0"/>
         <v>23.733238400379729</v>
       </c>
@@ -8228,10 +8228,10 @@
       <c r="C13" s="42">
         <v>120</v>
       </c>
-      <c r="D13" s="130">
+      <c r="D13" s="91">
         <v>1.72</v>
       </c>
-      <c r="E13" s="130">
+      <c r="E13" s="91">
         <f t="shared" si="0"/>
         <v>40.562466197944836</v>
       </c>
@@ -8261,12 +8261,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="97" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
@@ -8459,16 +8459,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="95" t="s">
+      <c r="A1" s="98" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
+      <c r="B1" s="98"/>
+      <c r="C1" s="98"/>
+      <c r="D1" s="98"/>
+      <c r="E1" s="98"/>
+      <c r="F1" s="98"/>
+      <c r="G1" s="98"/>
+      <c r="H1" s="98"/>
     </row>
     <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="23" t="s">
@@ -8732,11 +8732,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="99" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
     </row>
     <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
@@ -8875,12 +8875,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="99" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
@@ -9041,11 +9041,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="100" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="98"/>
-      <c r="C1" s="99"/>
+      <c r="B1" s="101"/>
+      <c r="C1" s="102"/>
     </row>
     <row r="2" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
@@ -9171,12 +9171,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="99" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">

</xml_diff>